<commit_message>
fix: enable temperature/top_p in LLM calls, add r3agentv3 agent and evaluation scripts
Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/libreoffice_calc_njc/27fdf845-4947-48cf-a282-8163a3941abf/Customer_Deduplicate.xlsx
+++ b/assets/libreoffice_calc_njc/27fdf845-4947-48cf-a282-8163a3941abf/Customer_Deduplicate.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="14">
   <si>
     <t xml:space="preserve">Customer Names with Duplicates</t>
   </si>
@@ -137,8 +137,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -160,138 +164,174 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:D26"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D2" s="0" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="D3" s="0" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="D4" s="0" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="D5" s="0" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="D6" s="0" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="D7" s="0" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="D8" s="0" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="D9" s="0" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="D10" s="0" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="D11" s="0" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="D12" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="D13" s="0" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>